<commit_message>
Sync revised supplementary materials: streamline S18/S19 and clarify frame endpoints
</commit_message>
<xml_diff>
--- a/supplementary-material/Supplementary Table S16.xlsx
+++ b/supplementary-material/Supplementary Table S16.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86CFC913-79BE-BA4F-9A7D-08BDAD288FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77152600-CBA5-664F-9A74-AC6E5AD47E6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20780" yWindow="6920" windowWidth="15960" windowHeight="18080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,29 +41,28 @@
     <font>
       <sz val="10"/>
       <color indexed="8"/>
-      <name val="Helvetica Neue"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="12"/>
       <color indexed="8"/>
-      <name val="Helvetica Neue"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color indexed="8"/>
-      <name val="Helvetica Neue"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="FangSong"/>
-      <family val="3"/>
-      <charset val="134"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -72,14 +71,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="9"/>
-        <bgColor auto="1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="12"/>
-        <bgColor auto="1"/>
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -209,19 +202,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -230,8 +214,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -361,12 +354,12 @@
     </a:clrScheme>
     <a:fontScheme name="Blank">
       <a:majorFont>
-        <a:latin typeface="Helvetica Neue"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface="Helvetica Neue"/>
         <a:cs typeface="Helvetica Neue"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Helvetica Neue"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface="Helvetica Neue"/>
         <a:cs typeface="Helvetica Neue"/>
       </a:minorFont>
@@ -1364,470 +1357,470 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C42"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.33203125" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.3984375" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.83203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="25.1640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="8.33203125" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.33203125" style="1"/>
+    <col min="2" max="2" width="4.796875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="25.19921875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="8.3984375" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.3984375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-    </row>
-    <row r="2" spans="1:3" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+    </row>
+    <row r="2" spans="1:3" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="6" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="3">
+    <row r="3" spans="1:3" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="8">
         <v>1</v>
       </c>
-      <c r="B3" s="4">
-        <v>20</v>
-      </c>
-      <c r="C3" s="5">
+      <c r="B3" s="2">
+        <v>20</v>
+      </c>
+      <c r="C3" s="3">
         <v>861</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="6">
+    <row r="4" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="9">
         <v>2</v>
       </c>
-      <c r="B4" s="7">
-        <v>20</v>
-      </c>
-      <c r="C4" s="8">
+      <c r="B4" s="4">
+        <v>20</v>
+      </c>
+      <c r="C4" s="5">
         <v>871</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="6">
+    <row r="5" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="9">
         <v>3</v>
       </c>
-      <c r="B5" s="7">
-        <v>20</v>
-      </c>
-      <c r="C5" s="8">
+      <c r="B5" s="4">
+        <v>20</v>
+      </c>
+      <c r="C5" s="5">
         <v>862</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="6">
+    <row r="6" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="9">
         <v>5</v>
       </c>
-      <c r="B6" s="7">
-        <v>20</v>
-      </c>
-      <c r="C6" s="8">
+      <c r="B6" s="4">
+        <v>20</v>
+      </c>
+      <c r="C6" s="5">
         <v>865</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="6">
+    <row r="7" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="9">
         <v>6</v>
       </c>
-      <c r="B7" s="7">
-        <v>20</v>
-      </c>
-      <c r="C7" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="6">
+      <c r="B7" s="4">
+        <v>20</v>
+      </c>
+      <c r="C7" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="9">
         <v>7</v>
       </c>
-      <c r="B8" s="7">
-        <v>20</v>
-      </c>
-      <c r="C8" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="6">
+      <c r="B8" s="4">
+        <v>20</v>
+      </c>
+      <c r="C8" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="9">
         <v>8</v>
       </c>
-      <c r="B9" s="7">
-        <v>20</v>
-      </c>
-      <c r="C9" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="6">
+      <c r="B9" s="4">
+        <v>20</v>
+      </c>
+      <c r="C9" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="9">
         <v>9</v>
       </c>
-      <c r="B10" s="7">
-        <v>20</v>
-      </c>
-      <c r="C10" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="6">
+      <c r="B10" s="4">
+        <v>20</v>
+      </c>
+      <c r="C10" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="9">
         <v>10</v>
       </c>
-      <c r="B11" s="7">
-        <v>20</v>
-      </c>
-      <c r="C11" s="8">
+      <c r="B11" s="4">
+        <v>20</v>
+      </c>
+      <c r="C11" s="5">
         <v>901</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="6">
+    <row r="12" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="9">
         <v>11</v>
       </c>
-      <c r="B12" s="7">
-        <v>20</v>
-      </c>
-      <c r="C12" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="6">
+      <c r="B12" s="4">
+        <v>20</v>
+      </c>
+      <c r="C12" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="9">
         <v>12</v>
       </c>
-      <c r="B13" s="7">
-        <v>20</v>
-      </c>
-      <c r="C13" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="6">
+      <c r="B13" s="4">
+        <v>20</v>
+      </c>
+      <c r="C13" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="9">
         <v>13</v>
       </c>
-      <c r="B14" s="7">
-        <v>20</v>
-      </c>
-      <c r="C14" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="6">
+      <c r="B14" s="4">
+        <v>20</v>
+      </c>
+      <c r="C14" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="9">
         <v>14</v>
       </c>
-      <c r="B15" s="7">
-        <v>20</v>
-      </c>
-      <c r="C15" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="6">
+      <c r="B15" s="4">
+        <v>20</v>
+      </c>
+      <c r="C15" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="9">
         <v>15</v>
       </c>
-      <c r="B16" s="7">
-        <v>20</v>
-      </c>
-      <c r="C16" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="6">
+      <c r="B16" s="4">
+        <v>20</v>
+      </c>
+      <c r="C16" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="9">
         <v>16</v>
       </c>
-      <c r="B17" s="7">
-        <v>20</v>
-      </c>
-      <c r="C17" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A18" s="6">
+      <c r="B17" s="4">
+        <v>20</v>
+      </c>
+      <c r="C17" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="9">
         <v>17</v>
       </c>
-      <c r="B18" s="7">
-        <v>20</v>
-      </c>
-      <c r="C18" s="8">
+      <c r="B18" s="4">
+        <v>20</v>
+      </c>
+      <c r="C18" s="5">
         <v>865</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A19" s="6">
+    <row r="19" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="9">
         <v>18</v>
       </c>
-      <c r="B19" s="7">
-        <v>20</v>
-      </c>
-      <c r="C19" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A20" s="6">
+      <c r="B19" s="4">
+        <v>20</v>
+      </c>
+      <c r="C19" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="9">
         <v>19</v>
       </c>
-      <c r="B20" s="7">
+      <c r="B20" s="4">
         <v>15</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20" s="5">
         <v>1010</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A21" s="6">
+    <row r="21" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="9">
         <v>90</v>
       </c>
-      <c r="B21" s="7">
-        <v>20</v>
-      </c>
-      <c r="C21" s="8">
+      <c r="B21" s="4">
+        <v>20</v>
+      </c>
+      <c r="C21" s="5">
         <v>888</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="6">
+    <row r="22" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="9">
         <v>91</v>
       </c>
-      <c r="B22" s="7">
-        <v>20</v>
-      </c>
-      <c r="C22" s="8">
+      <c r="B22" s="4">
+        <v>20</v>
+      </c>
+      <c r="C22" s="5">
         <v>871</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A23" s="6">
+    <row r="23" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="9">
         <v>92</v>
       </c>
-      <c r="B23" s="7">
-        <v>20</v>
-      </c>
-      <c r="C23" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A24" s="6">
+      <c r="B23" s="4">
+        <v>20</v>
+      </c>
+      <c r="C23" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="9">
         <v>93</v>
       </c>
-      <c r="B24" s="7">
-        <v>20</v>
-      </c>
-      <c r="C24" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A25" s="6">
+      <c r="B24" s="4">
+        <v>20</v>
+      </c>
+      <c r="C24" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="9">
         <v>94</v>
       </c>
-      <c r="B25" s="7">
-        <v>20</v>
-      </c>
-      <c r="C25" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A26" s="6">
+      <c r="B25" s="4">
+        <v>20</v>
+      </c>
+      <c r="C25" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="9">
         <v>95</v>
       </c>
-      <c r="B26" s="7">
-        <v>20</v>
-      </c>
-      <c r="C26" s="8">
+      <c r="B26" s="4">
+        <v>20</v>
+      </c>
+      <c r="C26" s="5">
         <v>887</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A27" s="6">
+    <row r="27" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="9">
         <v>96</v>
       </c>
-      <c r="B27" s="7">
-        <v>20</v>
-      </c>
-      <c r="C27" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A28" s="6">
+      <c r="B27" s="4">
+        <v>20</v>
+      </c>
+      <c r="C27" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="9">
         <v>97</v>
       </c>
-      <c r="B28" s="7">
-        <v>20</v>
-      </c>
-      <c r="C28" s="8">
+      <c r="B28" s="4">
+        <v>20</v>
+      </c>
+      <c r="C28" s="5">
         <v>859</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A29" s="6">
+    <row r="29" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="9">
         <v>98</v>
       </c>
-      <c r="B29" s="7">
-        <v>20</v>
-      </c>
-      <c r="C29" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A30" s="6">
+      <c r="B29" s="4">
+        <v>20</v>
+      </c>
+      <c r="C29" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="9">
         <v>99</v>
       </c>
-      <c r="B30" s="7">
-        <v>20</v>
-      </c>
-      <c r="C30" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A31" s="6">
+      <c r="B30" s="4">
+        <v>20</v>
+      </c>
+      <c r="C30" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="9">
         <v>100</v>
       </c>
-      <c r="B31" s="7">
-        <v>20</v>
-      </c>
-      <c r="C31" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A32" s="6">
+      <c r="B31" s="4">
+        <v>20</v>
+      </c>
+      <c r="C31" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="9">
         <v>101</v>
       </c>
-      <c r="B32" s="7">
-        <v>20</v>
-      </c>
-      <c r="C32" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A33" s="6">
+      <c r="B32" s="4">
+        <v>20</v>
+      </c>
+      <c r="C32" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="9">
         <v>102</v>
       </c>
-      <c r="B33" s="7">
-        <v>20</v>
-      </c>
-      <c r="C33" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A34" s="6">
+      <c r="B33" s="4">
+        <v>20</v>
+      </c>
+      <c r="C33" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="9">
         <v>103</v>
       </c>
-      <c r="B34" s="7">
-        <v>20</v>
-      </c>
-      <c r="C34" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A35" s="6">
+      <c r="B34" s="4">
+        <v>20</v>
+      </c>
+      <c r="C34" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="9">
         <v>104</v>
       </c>
-      <c r="B35" s="7">
-        <v>20</v>
-      </c>
-      <c r="C35" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A36" s="6">
+      <c r="B35" s="4">
+        <v>20</v>
+      </c>
+      <c r="C35" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="9">
         <v>105</v>
       </c>
-      <c r="B36" s="7">
-        <v>20</v>
-      </c>
-      <c r="C36" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A37" s="6">
+      <c r="B36" s="4">
+        <v>20</v>
+      </c>
+      <c r="C36" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="9">
         <v>106</v>
       </c>
-      <c r="B37" s="7">
-        <v>20</v>
-      </c>
-      <c r="C37" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A38" s="6">
+      <c r="B37" s="4">
+        <v>20</v>
+      </c>
+      <c r="C37" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="9">
         <v>107</v>
       </c>
-      <c r="B38" s="7">
-        <v>20</v>
-      </c>
-      <c r="C38" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A39" s="6">
+      <c r="B38" s="4">
+        <v>20</v>
+      </c>
+      <c r="C38" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="9">
         <v>108</v>
       </c>
-      <c r="B39" s="7">
-        <v>20</v>
-      </c>
-      <c r="C39" s="8">
-        <v>863</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A40" s="6">
+      <c r="B39" s="4">
+        <v>20</v>
+      </c>
+      <c r="C39" s="5">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="9">
         <v>109</v>
       </c>
-      <c r="B40" s="7">
-        <v>20</v>
-      </c>
-      <c r="C40" s="8">
+      <c r="B40" s="4">
+        <v>20</v>
+      </c>
+      <c r="C40" s="5">
         <v>861</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A41" s="6">
+    <row r="41" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="9">
         <v>110</v>
       </c>
-      <c r="B41" s="7">
-        <v>20</v>
-      </c>
-      <c r="C41" s="8">
+      <c r="B41" s="4">
+        <v>20</v>
+      </c>
+      <c r="C41" s="5">
         <v>887</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A42" s="6">
+    <row r="42" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="9">
         <v>111</v>
       </c>
-      <c r="B42" s="7">
-        <v>20</v>
-      </c>
-      <c r="C42" s="8">
+      <c r="B42" s="4">
+        <v>20</v>
+      </c>
+      <c r="C42" s="5">
         <v>863</v>
       </c>
     </row>
@@ -1839,7 +1832,7 @@
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup orientation="portrait"/>
   <headerFooter>
-    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
+    <oddFooter>&amp;C&amp;"Calibri,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>